<commit_message>
Add marketing/sales track to the launch WBS
The plan had no positioning or outreach work — one line about "listing
monitor candidates" was the entire go-to-market. With invites running
through a well-connected team member, positioning now has to exist
before there's anything to hand them: it feeds both the sales one-pager
and the LP copy, so both wait on it explicitly.

Renumbers the product/monitor/billing categories to make room.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/service-launch-wbs.xlsx
+++ b/docs/service-launch-wbs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Satoshi Sudo\AppData\Local\Temp\claude\C--Users-Satoshi-Sudo--claude\56290f08-2ae4-4b65-b5a1-b34dcffeeb19\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C3BFA70-0D8A-476E-832B-B6E176168D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7F4CD8-2D5A-4E07-9B5E-D2822B6570C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19110" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="253">
   <si>
     <t>THE CONCIERGE　サービス開始WBS</t>
   </si>
@@ -294,12 +294,15 @@
     <t>LP（ホームページ）を制作・公開</t>
   </si>
   <si>
-    <t>独自ドメイン上で機能を説明し、プライバシーポリシーへリンクしている</t>
+    <t>独自ドメイン上で機能を説明し、プライバシーポリシーへリンクしている。訴求文言は3.1のポジショニングと揃っている</t>
   </si>
   <si>
     <t>自分/開発</t>
   </si>
   <si>
+    <t>2.3,3.1</t>
+  </si>
+  <si>
     <t>2.7</t>
   </si>
   <si>
@@ -366,7 +369,31 @@
     <t>3.1</t>
   </si>
   <si>
-    <t>3 プロダクト</t>
+    <t>3 マーケ・営業資料</t>
+  </si>
+  <si>
+    <t>ポジショニング・ターゲット・訴求メッセージを確定</t>
+  </si>
+  <si>
+    <t>「誰に／何を／なぜ今」が1枚にまとまり、LP・営業資料の共通言語になっている（既存の投資家向けpositioning.htmlを土台に招待制モニター向けへ転用）</t>
+  </si>
+  <si>
+    <t>自分/チーム</t>
+  </si>
+  <si>
+    <t>3.2</t>
+  </si>
+  <si>
+    <t>招待用の営業資料（1枚もの＋声かけトークポイント）を作成</t>
+  </si>
+  <si>
+    <t>人脈を持つメンバーがそのまま送れる資料（サービス概要・画面・招待条件・声かけ文面）が完成している</t>
+  </si>
+  <si>
+    <t>4.1</t>
+  </si>
+  <si>
+    <t>4 プロダクト</t>
   </si>
   <si>
     <t>旧Vercelプロジェクト（the-concierge-delta）を削除</t>
@@ -375,7 +402,7 @@
     <t>誤アクセスの原因を除去</t>
   </si>
   <si>
-    <t>3.2</t>
+    <t>4.2</t>
   </si>
   <si>
     <t>4人ドッグフーディング（2週間）</t>
@@ -387,7 +414,7 @@
     <t>全員</t>
   </si>
   <si>
-    <t>3.3</t>
+    <t>4.3</t>
   </si>
   <si>
     <t>不具合修正・改善（テスト結果の反映）</t>
@@ -396,7 +423,7 @@
     <t>重大な不具合がゼロ。モニターに出せる品質</t>
   </si>
   <si>
-    <t>3.4</t>
+    <t>4.4</t>
   </si>
   <si>
     <t>エラー監視の導入（Sentry等）</t>
@@ -405,7 +432,7 @@
     <t>本番エラーが自動で通知される。モニター中の障害検知に必須</t>
   </si>
   <si>
-    <t>3.5</t>
+    <t>4.5</t>
   </si>
   <si>
     <t>Outlook連携の復旧（Azure設定）</t>
@@ -414,7 +441,7 @@
     <t>Outlookユーザーが連携できる。法人層には必要</t>
   </si>
   <si>
-    <t>3.6</t>
+    <t>4.6</t>
   </si>
   <si>
     <t>プロンプトキャッシングでAPI費用を削減</t>
@@ -423,7 +450,7 @@
     <t>システムプロンプトを再構成し、キャッシュが効いている</t>
   </si>
   <si>
-    <t>3.7</t>
+    <t>4.7</t>
   </si>
   <si>
     <t>モニター向けオンボーディングの改善</t>
@@ -432,7 +459,7 @@
     <t>説明なしで初回設定を完了できる</t>
   </si>
   <si>
-    <t>3.8</t>
+    <t>4.8</t>
   </si>
   <si>
     <t>利用状況の可視化（誰が何回使ったか）</t>
@@ -441,7 +468,7 @@
     <t>継続率と利用頻度を数字で追える</t>
   </si>
   <si>
-    <t>3.9</t>
+    <t>4.9</t>
   </si>
   <si>
     <t>バックアップ・障害時の復旧手順を用意</t>
@@ -450,10 +477,10 @@
     <t>DBバックアップが自動化され、復旧手順が文書化されている</t>
   </si>
   <si>
-    <t>4.1</t>
-  </si>
-  <si>
-    <t>4 モニター運用</t>
+    <t>5.1</t>
+  </si>
+  <si>
+    <t>5 モニター運用</t>
   </si>
   <si>
     <t>モニター募集要項・条件を確定</t>
@@ -462,25 +489,34 @@
     <t>提供内容・期間・料金（無料/低額）・フィードバック義務を明文化</t>
   </si>
   <si>
-    <t>4.2</t>
-  </si>
-  <si>
-    <t>申込フォーム・招待メール文面を用意</t>
-  </si>
-  <si>
-    <t>申込〜利用開始までの導線が完成</t>
-  </si>
-  <si>
-    <t>4.3</t>
-  </si>
-  <si>
-    <t>モニター候補のリストアップ・打診</t>
-  </si>
-  <si>
-    <t>開始時に必要な人数の内諾が取れている</t>
-  </si>
-  <si>
-    <t>4.4</t>
+    <t>5.2</t>
+  </si>
+  <si>
+    <t>申込フォーム・正式な招待メール文面を用意（申込導線）</t>
+  </si>
+  <si>
+    <t>申込〜利用開始までの導線が完成。3.1のメッセージと表現がそろっている</t>
+  </si>
+  <si>
+    <t>3.1,5.1</t>
+  </si>
+  <si>
+    <t>5.3</t>
+  </si>
+  <si>
+    <t>モニター候補のリストアップ・打診（人脈メンバー中心）</t>
+  </si>
+  <si>
+    <t>開始時に必要な人数の内諾が取れている。3.2の営業資料を使って声かけする</t>
+  </si>
+  <si>
+    <t>自分/人脈メンバー</t>
+  </si>
+  <si>
+    <t>3.2,5.1</t>
+  </si>
+  <si>
+    <t>5.4</t>
   </si>
   <si>
     <t>★モニター開始（招待制・〜100名）</t>
@@ -489,10 +525,10 @@
     <t>招待した方が実際に使い始めている</t>
   </si>
   <si>
-    <t>3.3,4.3</t>
-  </si>
-  <si>
-    <t>4.5</t>
+    <t>4.3,5.3</t>
+  </si>
+  <si>
+    <t>5.5</t>
   </si>
   <si>
     <t>テストユーザー登録の運用</t>
@@ -501,7 +537,7 @@
     <t>申込ごとにGoogle側へ登録する手順が回っている</t>
   </si>
   <si>
-    <t>4.6</t>
+    <t>5.6</t>
   </si>
   <si>
     <t>サポート窓口の設置・運用</t>
@@ -510,7 +546,7 @@
     <t>問い合わせ先が公開され、返信の担当と目安時間が決まっている</t>
   </si>
   <si>
-    <t>4.7</t>
+    <t>5.7</t>
   </si>
   <si>
     <t>週次でフィードバック収集・改善反映</t>
@@ -519,7 +555,7 @@
     <t>毎週の改善サイクルが回っている</t>
   </si>
   <si>
-    <t>4.8</t>
+    <t>5.8</t>
   </si>
   <si>
     <t>KPI計測（継続率・利用頻度・音声利用率）</t>
@@ -528,13 +564,13 @@
     <t>有料化の判断材料になる数字が揃っている</t>
   </si>
   <si>
-    <t>3.8,4.4</t>
-  </si>
-  <si>
-    <t>5.1</t>
-  </si>
-  <si>
-    <t>5 有料化準備</t>
+    <t>4.8,5.4</t>
+  </si>
+  <si>
+    <t>6.1</t>
+  </si>
+  <si>
+    <t>6 有料化準備</t>
   </si>
   <si>
     <t>料金プランを確定</t>
@@ -543,7 +579,7 @@
     <t>プラン構成と価格が決定（要件書は¥5,000/¥8,000/法人¥40,000想定）</t>
   </si>
   <si>
-    <t>5.2</t>
+    <t>6.2</t>
   </si>
   <si>
     <t>特定商取引法に基づく表記を作成</t>
@@ -552,10 +588,10 @@
     <t>事業者名・所在地・連絡先・解約条件をサイトに掲載</t>
   </si>
   <si>
-    <t>1.8,5.1</t>
-  </si>
-  <si>
-    <t>5.3</t>
+    <t>1.8,6.1</t>
+  </si>
+  <si>
+    <t>6.3</t>
   </si>
   <si>
     <t>Stripe アカウント開設</t>
@@ -564,7 +600,7 @@
     <t>法人口座を登録し、入金確認まで完了</t>
   </si>
   <si>
-    <t>5.4</t>
+    <t>6.4</t>
   </si>
   <si>
     <t>課金機能の実装（10月）</t>
@@ -573,7 +609,7 @@
     <t>サブスク登録・解約・failed payment の処理が動く</t>
   </si>
   <si>
-    <t>5.5</t>
+    <t>6.5</t>
   </si>
   <si>
     <t>請求・領収書の運用設計（10月）</t>
@@ -618,10 +654,10 @@
     <t>8/13</t>
   </si>
   <si>
-    <t>商号を確定</t>
-  </si>
-  <si>
-    <t>プライバシーポリシー・利用規約・ドメインがここで止まる</t>
+    <t>商号・ポジショニングを確定</t>
+  </si>
+  <si>
+    <t>プライバシーポリシー・利用規約・ドメイン・LP訴求・営業資料がすべてここで止まる</t>
   </si>
   <si>
     <t>8/25</t>
@@ -751,6 +787,15 @@
   </si>
   <si>
     <t>定款・登記・ポリシーは専門家に外注し、自分は開発と審査対応に集中する</t>
+  </si>
+  <si>
+    <t>招待の集客が特定1名の人脈に集中している</t>
+  </si>
+  <si>
+    <t>チーム内の人脈を持つ1名の稼働・都合に依存しており、その人が動けないと100名という目標に届かない</t>
+  </si>
+  <si>
+    <t>8月中に営業資料（3.2）を用意して早期に声かけを開始してもらう。他の3名にも並行して自分の人脈への打診を依頼し、一極集中を避ける</t>
   </si>
   <si>
     <t>※ 会社設立・税務・法務・商標に関する記載は一般的な流れの整理です。実際の手続きは司法書士・税理士・弁理士にご確認ください。</t>
@@ -1327,7 +1372,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R57"/>
+  <dimension ref="A1:R59"/>
   <sheetFormatPr defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1482,7 +1527,7 @@
         <v>46247</v>
       </c>
       <c r="H6" s="12">
-        <f t="shared" ref="H6:H50" si="0">G6-F6+1</f>
+        <f t="shared" ref="H6:H52" si="0">G6-F6+1</f>
         <v>3</v>
       </c>
       <c r="I6" s="8" t="s">
@@ -2115,7 +2160,7 @@
       <c r="Q21" s="14"/>
       <c r="R21" s="14"/>
     </row>
-    <row r="22" spans="1:18" ht="30">
+    <row r="22" spans="1:18" ht="45">
       <c r="A22" s="8" t="s">
         <v>82</v>
       </c>
@@ -2142,7 +2187,7 @@
         <v>8</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="J22" s="8" t="s">
         <v>30</v>
@@ -2158,19 +2203,19 @@
     </row>
     <row r="23" spans="1:18" ht="30">
       <c r="A23" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B23" s="9" t="s">
         <v>66</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F23" s="11">
         <v>46251</v>
@@ -2199,19 +2244,19 @@
     </row>
     <row r="24" spans="1:18" ht="15">
       <c r="A24" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B24" s="9" t="s">
         <v>66</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F24" s="11">
         <v>46251</v>
@@ -2240,16 +2285,16 @@
     </row>
     <row r="25" spans="1:18" ht="30">
       <c r="A25" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B25" s="9" t="s">
         <v>66</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E25" s="8" t="s">
         <v>28</v>
@@ -2265,7 +2310,7 @@
         <v>4</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J25" s="8" t="s">
         <v>30</v>
@@ -2281,16 +2326,16 @@
     </row>
     <row r="26" spans="1:18" ht="15">
       <c r="A26" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B26" s="9" t="s">
         <v>66</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>28</v>
@@ -2322,16 +2367,16 @@
     </row>
     <row r="27" spans="1:18" ht="15">
       <c r="A27" s="16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B27" s="17" t="s">
         <v>66</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E27" s="16" t="s">
         <v>28</v>
@@ -2347,7 +2392,7 @@
         <v>1</v>
       </c>
       <c r="I27" s="16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J27" s="16" t="s">
         <v>30</v>
@@ -2363,16 +2408,16 @@
     </row>
     <row r="28" spans="1:18" ht="30">
       <c r="A28" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B28" s="9" t="s">
         <v>66</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E28" s="8" t="s">
         <v>28</v>
@@ -2388,7 +2433,7 @@
         <v>31</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J28" s="8" t="s">
         <v>30</v>
@@ -2402,31 +2447,31 @@
       <c r="Q28" s="13"/>
       <c r="R28" s="13"/>
     </row>
-    <row r="29" spans="1:18" ht="15">
+    <row r="29" spans="1:18" ht="45">
       <c r="A29" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>28</v>
+        <v>112</v>
       </c>
       <c r="F29" s="11">
         <v>46245</v>
       </c>
       <c r="G29" s="11">
-        <v>46245</v>
+        <v>46247</v>
       </c>
       <c r="H29" s="12">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>29</v>
@@ -2434,7 +2479,7 @@
       <c r="J29" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="K29" s="15"/>
+      <c r="K29" s="13"/>
       <c r="L29" s="14"/>
       <c r="M29" s="14"/>
       <c r="N29" s="14"/>
@@ -2445,39 +2490,39 @@
     </row>
     <row r="30" spans="1:18" ht="30">
       <c r="A30" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B30" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F30" s="11">
+        <v>46248</v>
+      </c>
+      <c r="G30" s="11">
+        <v>46253</v>
+      </c>
+      <c r="H30" s="12">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="I30" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="C30" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="D30" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="F30" s="11">
-        <v>46245</v>
-      </c>
-      <c r="G30" s="11">
-        <v>46258</v>
-      </c>
-      <c r="H30" s="12">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="I30" s="8" t="s">
-        <v>65</v>
-      </c>
       <c r="J30" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="K30" s="15"/>
-      <c r="L30" s="15"/>
-      <c r="M30" s="15"/>
+      <c r="K30" s="13"/>
+      <c r="L30" s="13"/>
+      <c r="M30" s="14"/>
       <c r="N30" s="14"/>
       <c r="O30" s="14"/>
       <c r="P30" s="14"/>
@@ -2486,39 +2531,39 @@
     </row>
     <row r="31" spans="1:18" ht="15">
       <c r="A31" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
       <c r="F31" s="11">
-        <v>46251</v>
+        <v>46245</v>
       </c>
       <c r="G31" s="11">
-        <v>46262</v>
+        <v>46245</v>
       </c>
       <c r="H31" s="12">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>111</v>
+        <v>29</v>
       </c>
       <c r="J31" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="K31" s="14"/>
-      <c r="L31" s="13"/>
-      <c r="M31" s="13"/>
+      <c r="K31" s="15"/>
+      <c r="L31" s="14"/>
+      <c r="M31" s="14"/>
       <c r="N31" s="14"/>
       <c r="O31" s="14"/>
       <c r="P31" s="14"/>
@@ -2527,39 +2572,39 @@
     </row>
     <row r="32" spans="1:18" ht="30">
       <c r="A32" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="F32" s="11">
-        <v>46251</v>
+        <v>46245</v>
       </c>
       <c r="G32" s="11">
-        <v>46253</v>
+        <v>46258</v>
       </c>
       <c r="H32" s="12">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="J32" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="K32" s="14"/>
+      <c r="K32" s="15"/>
       <c r="L32" s="15"/>
-      <c r="M32" s="14"/>
+      <c r="M32" s="15"/>
       <c r="N32" s="14"/>
       <c r="O32" s="14"/>
       <c r="P32" s="14"/>
@@ -2568,70 +2613,70 @@
     </row>
     <row r="33" spans="1:18" ht="15">
       <c r="A33" s="8" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="F33" s="11">
-        <v>46253</v>
+        <v>46251</v>
       </c>
       <c r="G33" s="11">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H33" s="12">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>29</v>
+        <v>120</v>
       </c>
       <c r="J33" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K33" s="14"/>
-      <c r="L33" s="15"/>
-      <c r="M33" s="15"/>
+      <c r="L33" s="13"/>
+      <c r="M33" s="13"/>
       <c r="N33" s="14"/>
       <c r="O33" s="14"/>
       <c r="P33" s="14"/>
       <c r="Q33" s="14"/>
       <c r="R33" s="14"/>
     </row>
-    <row r="34" spans="1:18" ht="15">
+    <row r="34" spans="1:18" ht="30">
       <c r="A34" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E34" s="8" t="s">
         <v>78</v>
       </c>
       <c r="F34" s="11">
-        <v>46260</v>
+        <v>46251</v>
       </c>
       <c r="G34" s="11">
-        <v>46261</v>
+        <v>46253</v>
       </c>
       <c r="H34" s="12">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I34" s="8" t="s">
         <v>29</v>
@@ -2640,8 +2685,8 @@
         <v>30</v>
       </c>
       <c r="K34" s="14"/>
-      <c r="L34" s="14"/>
-      <c r="M34" s="15"/>
+      <c r="L34" s="15"/>
+      <c r="M34" s="14"/>
       <c r="N34" s="14"/>
       <c r="O34" s="14"/>
       <c r="P34" s="14"/>
@@ -2650,38 +2695,38 @@
     </row>
     <row r="35" spans="1:18" ht="15">
       <c r="A35" s="8" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="F35" s="11">
-        <v>46258</v>
+        <v>46253</v>
       </c>
       <c r="G35" s="11">
-        <v>46262</v>
+        <v>46260</v>
       </c>
       <c r="H35" s="12">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>111</v>
+        <v>29</v>
       </c>
       <c r="J35" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K35" s="14"/>
-      <c r="L35" s="14"/>
+      <c r="L35" s="15"/>
       <c r="M35" s="15"/>
       <c r="N35" s="14"/>
       <c r="O35" s="14"/>
@@ -2691,29 +2736,29 @@
     </row>
     <row r="36" spans="1:18" ht="15">
       <c r="A36" s="8" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E36" s="8" t="s">
         <v>78</v>
       </c>
       <c r="F36" s="11">
-        <v>46258</v>
+        <v>46260</v>
       </c>
       <c r="G36" s="11">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="H36" s="12">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I36" s="8" t="s">
         <v>29</v>
@@ -2730,62 +2775,62 @@
       <c r="Q36" s="14"/>
       <c r="R36" s="14"/>
     </row>
-    <row r="37" spans="1:18" ht="30">
+    <row r="37" spans="1:18" ht="15">
       <c r="A37" s="8" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="E37" s="8" t="s">
         <v>78</v>
       </c>
       <c r="F37" s="11">
-        <v>46266</v>
+        <v>46258</v>
       </c>
       <c r="G37" s="11">
-        <v>46269</v>
+        <v>46262</v>
       </c>
       <c r="H37" s="12">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>29</v>
+        <v>120</v>
       </c>
       <c r="J37" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K37" s="14"/>
       <c r="L37" s="14"/>
-      <c r="M37" s="14"/>
-      <c r="N37" s="15"/>
+      <c r="M37" s="15"/>
+      <c r="N37" s="14"/>
       <c r="O37" s="14"/>
       <c r="P37" s="14"/>
       <c r="Q37" s="14"/>
       <c r="R37" s="14"/>
     </row>
-    <row r="38" spans="1:18" ht="30">
+    <row r="38" spans="1:18" ht="15">
       <c r="A38" s="8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>137</v>
+        <v>117</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="F38" s="11">
         <v>46258</v>
@@ -2812,59 +2857,59 @@
       <c r="Q38" s="14"/>
       <c r="R38" s="14"/>
     </row>
-    <row r="39" spans="1:18" ht="15">
+    <row r="39" spans="1:18" ht="30">
       <c r="A39" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>137</v>
+        <v>117</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="F39" s="11">
-        <v>46260</v>
+        <v>46266</v>
       </c>
       <c r="G39" s="11">
-        <v>46265</v>
+        <v>46269</v>
       </c>
       <c r="H39" s="12">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>136</v>
+        <v>29</v>
       </c>
       <c r="J39" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K39" s="14"/>
       <c r="L39" s="14"/>
-      <c r="M39" s="15"/>
+      <c r="M39" s="14"/>
       <c r="N39" s="15"/>
       <c r="O39" s="14"/>
       <c r="P39" s="14"/>
       <c r="Q39" s="14"/>
       <c r="R39" s="14"/>
     </row>
-    <row r="40" spans="1:18" ht="15">
+    <row r="40" spans="1:18" ht="30">
       <c r="A40" s="8" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="E40" s="8" t="s">
         <v>28</v>
@@ -2873,165 +2918,165 @@
         <v>46258</v>
       </c>
       <c r="G40" s="11">
-        <v>46265</v>
+        <v>46262</v>
       </c>
       <c r="H40" s="12">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I40" s="8" t="s">
-        <v>136</v>
+        <v>29</v>
       </c>
       <c r="J40" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K40" s="14"/>
       <c r="L40" s="14"/>
-      <c r="M40" s="13"/>
-      <c r="N40" s="13"/>
+      <c r="M40" s="15"/>
+      <c r="N40" s="14"/>
       <c r="O40" s="14"/>
       <c r="P40" s="14"/>
       <c r="Q40" s="14"/>
       <c r="R40" s="14"/>
     </row>
-    <row r="41" spans="1:18" ht="15">
-      <c r="A41" s="16" t="s">
+    <row r="41" spans="1:18" ht="30">
+      <c r="A41" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B41" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="B41" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="C41" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="D41" s="18" t="s">
-        <v>148</v>
-      </c>
-      <c r="E41" s="16" t="s">
+      <c r="C41" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="E41" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F41" s="19">
-        <v>46266</v>
-      </c>
-      <c r="G41" s="19">
-        <v>46266</v>
-      </c>
-      <c r="H41" s="20">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="I41" s="16" t="s">
-        <v>149</v>
-      </c>
-      <c r="J41" s="16" t="s">
+      <c r="F41" s="11">
+        <v>46260</v>
+      </c>
+      <c r="G41" s="11">
+        <v>46265</v>
+      </c>
+      <c r="H41" s="12">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="I41" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="J41" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K41" s="14"/>
       <c r="L41" s="14"/>
-      <c r="M41" s="14"/>
-      <c r="N41" s="21"/>
+      <c r="M41" s="15"/>
+      <c r="N41" s="15"/>
       <c r="O41" s="14"/>
       <c r="P41" s="14"/>
       <c r="Q41" s="14"/>
       <c r="R41" s="14"/>
     </row>
-    <row r="42" spans="1:18" ht="15">
+    <row r="42" spans="1:18" ht="30">
       <c r="A42" s="8" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E42" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="F42" s="11">
+        <v>46254</v>
+      </c>
+      <c r="G42" s="11">
+        <v>46265</v>
+      </c>
+      <c r="H42" s="12">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="I42" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="J42" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="K42" s="14"/>
+      <c r="L42" s="13"/>
+      <c r="M42" s="13"/>
+      <c r="N42" s="13"/>
+      <c r="O42" s="14"/>
+      <c r="P42" s="14"/>
+      <c r="Q42" s="14"/>
+      <c r="R42" s="14"/>
+    </row>
+    <row r="43" spans="1:18" ht="15">
+      <c r="A43" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="C43" s="18" t="s">
+        <v>159</v>
+      </c>
+      <c r="D43" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="E43" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="F42" s="11">
+      <c r="F43" s="19">
         <v>46266</v>
       </c>
-      <c r="G42" s="11">
-        <v>46295</v>
-      </c>
-      <c r="H42" s="12">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-      <c r="I42" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="J42" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="K42" s="14"/>
-      <c r="L42" s="14"/>
-      <c r="M42" s="14"/>
-      <c r="N42" s="15"/>
-      <c r="O42" s="15"/>
-      <c r="P42" s="15"/>
-      <c r="Q42" s="15"/>
-      <c r="R42" s="15"/>
-    </row>
-    <row r="43" spans="1:18" ht="30">
-      <c r="A43" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="B43" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="C43" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="E43" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="F43" s="11">
+      <c r="G43" s="19">
         <v>46266</v>
       </c>
-      <c r="G43" s="11">
-        <v>46295</v>
-      </c>
-      <c r="H43" s="12">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-      <c r="I43" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="J43" s="8" t="s">
+      <c r="H43" s="20">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="I43" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="J43" s="16" t="s">
         <v>30</v>
       </c>
       <c r="K43" s="14"/>
       <c r="L43" s="14"/>
       <c r="M43" s="14"/>
-      <c r="N43" s="15"/>
-      <c r="O43" s="15"/>
-      <c r="P43" s="15"/>
-      <c r="Q43" s="15"/>
-      <c r="R43" s="15"/>
+      <c r="N43" s="21"/>
+      <c r="O43" s="14"/>
+      <c r="P43" s="14"/>
+      <c r="Q43" s="14"/>
+      <c r="R43" s="14"/>
     </row>
     <row r="44" spans="1:18" ht="15">
       <c r="A44" s="8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>114</v>
+        <v>28</v>
       </c>
       <c r="F44" s="11">
         <v>46266</v>
@@ -3044,7 +3089,7 @@
         <v>30</v>
       </c>
       <c r="I44" s="8" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="J44" s="8" t="s">
         <v>30</v>
@@ -3058,34 +3103,34 @@
       <c r="Q44" s="15"/>
       <c r="R44" s="15"/>
     </row>
-    <row r="45" spans="1:18" ht="15">
+    <row r="45" spans="1:18" ht="30">
       <c r="A45" s="8" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="E45" s="8" t="s">
         <v>28</v>
       </c>
       <c r="F45" s="11">
-        <v>46272</v>
+        <v>46266</v>
       </c>
       <c r="G45" s="11">
         <v>46295</v>
       </c>
       <c r="H45" s="12">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="J45" s="8" t="s">
         <v>30</v>
@@ -3093,40 +3138,40 @@
       <c r="K45" s="14"/>
       <c r="L45" s="14"/>
       <c r="M45" s="14"/>
-      <c r="N45" s="14"/>
+      <c r="N45" s="15"/>
       <c r="O45" s="15"/>
       <c r="P45" s="15"/>
       <c r="Q45" s="15"/>
       <c r="R45" s="15"/>
     </row>
-    <row r="46" spans="1:18" ht="30">
+    <row r="46" spans="1:18" ht="15">
       <c r="A46" s="8" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>28</v>
+        <v>123</v>
       </c>
       <c r="F46" s="11">
-        <v>46272</v>
+        <v>46266</v>
       </c>
       <c r="G46" s="11">
-        <v>46283</v>
+        <v>46295</v>
       </c>
       <c r="H46" s="12">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="I46" s="8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J46" s="8" t="s">
         <v>30</v>
@@ -3134,40 +3179,40 @@
       <c r="K46" s="14"/>
       <c r="L46" s="14"/>
       <c r="M46" s="14"/>
-      <c r="N46" s="14"/>
+      <c r="N46" s="15"/>
       <c r="O46" s="15"/>
       <c r="P46" s="15"/>
-      <c r="Q46" s="14"/>
-      <c r="R46" s="14"/>
+      <c r="Q46" s="15"/>
+      <c r="R46" s="15"/>
     </row>
     <row r="47" spans="1:18" ht="15">
       <c r="A47" s="8" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="E47" s="8" t="s">
         <v>28</v>
       </c>
       <c r="F47" s="11">
-        <v>46279</v>
+        <v>46272</v>
       </c>
       <c r="G47" s="11">
-        <v>46290</v>
+        <v>46295</v>
       </c>
       <c r="H47" s="12">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="J47" s="8" t="s">
         <v>30</v>
@@ -3176,39 +3221,39 @@
       <c r="L47" s="14"/>
       <c r="M47" s="14"/>
       <c r="N47" s="14"/>
-      <c r="O47" s="14"/>
+      <c r="O47" s="15"/>
       <c r="P47" s="15"/>
       <c r="Q47" s="15"/>
-      <c r="R47" s="14"/>
-    </row>
-    <row r="48" spans="1:18" ht="15">
+      <c r="R47" s="15"/>
+    </row>
+    <row r="48" spans="1:18" ht="30">
       <c r="A48" s="8" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="E48" s="8" t="s">
         <v>28</v>
       </c>
       <c r="F48" s="11">
-        <v>46293</v>
+        <v>46272</v>
       </c>
       <c r="G48" s="11">
-        <v>46295</v>
+        <v>46283</v>
       </c>
       <c r="H48" s="12">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="I48" s="8" t="s">
-        <v>59</v>
+        <v>171</v>
       </c>
       <c r="J48" s="8" t="s">
         <v>30</v>
@@ -3217,41 +3262,41 @@
       <c r="L48" s="14"/>
       <c r="M48" s="14"/>
       <c r="N48" s="14"/>
-      <c r="O48" s="14"/>
-      <c r="P48" s="14"/>
+      <c r="O48" s="15"/>
+      <c r="P48" s="15"/>
       <c r="Q48" s="14"/>
-      <c r="R48" s="15"/>
+      <c r="R48" s="14"/>
     </row>
     <row r="49" spans="1:18" ht="15">
-      <c r="A49" s="22" t="s">
-        <v>174</v>
-      </c>
-      <c r="B49" s="23" t="s">
-        <v>164</v>
-      </c>
-      <c r="C49" s="24" t="s">
-        <v>175</v>
-      </c>
-      <c r="D49" s="24" t="s">
+      <c r="A49" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B49" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="E49" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="F49" s="25">
-        <v>46296</v>
-      </c>
-      <c r="G49" s="25">
-        <v>46310</v>
+      <c r="C49" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="D49" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="E49" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F49" s="11">
+        <v>46279</v>
+      </c>
+      <c r="G49" s="11">
+        <v>46290</v>
       </c>
       <c r="H49" s="12">
         <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="I49" s="22" t="s">
-        <v>171</v>
-      </c>
-      <c r="J49" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="I49" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="J49" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K49" s="14"/>
@@ -3259,40 +3304,40 @@
       <c r="M49" s="14"/>
       <c r="N49" s="14"/>
       <c r="O49" s="14"/>
-      <c r="P49" s="14"/>
-      <c r="Q49" s="14"/>
-      <c r="R49" s="26"/>
+      <c r="P49" s="15"/>
+      <c r="Q49" s="15"/>
+      <c r="R49" s="14"/>
     </row>
     <row r="50" spans="1:18" ht="15">
-      <c r="A50" s="22" t="s">
-        <v>177</v>
-      </c>
-      <c r="B50" s="23" t="s">
-        <v>164</v>
-      </c>
-      <c r="C50" s="24" t="s">
-        <v>178</v>
-      </c>
-      <c r="D50" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="E50" s="22" t="s">
+      <c r="A50" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="D50" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="E50" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F50" s="25">
-        <v>46296</v>
-      </c>
-      <c r="G50" s="25">
-        <v>46310</v>
+      <c r="F50" s="11">
+        <v>46293</v>
+      </c>
+      <c r="G50" s="11">
+        <v>46295</v>
       </c>
       <c r="H50" s="12">
         <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="I50" s="22" t="s">
-        <v>171</v>
-      </c>
-      <c r="J50" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="I50" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="J50" s="8" t="s">
         <v>30</v>
       </c>
       <c r="K50" s="14"/>
@@ -3302,55 +3347,137 @@
       <c r="O50" s="14"/>
       <c r="P50" s="14"/>
       <c r="Q50" s="14"/>
-      <c r="R50" s="26"/>
-    </row>
-    <row r="52" spans="1:18" ht="18">
-      <c r="B52" s="27" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="53" spans="1:18" ht="15.5">
-      <c r="B53" s="28" t="s">
-        <v>181</v>
-      </c>
-      <c r="C53" s="29">
-        <f>COUNTA(A6:A50)</f>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="54" spans="1:18" ht="15.5">
-      <c r="B54" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="C54" s="29">
-        <f>COUNTIF(J6:J50,"未着手")</f>
-        <v>45</v>
+      <c r="R50" s="15"/>
+    </row>
+    <row r="51" spans="1:18" ht="15">
+      <c r="A51" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="B51" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="C51" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="D51" s="24" t="s">
+        <v>188</v>
+      </c>
+      <c r="E51" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="F51" s="25">
+        <v>46296</v>
+      </c>
+      <c r="G51" s="25">
+        <v>46310</v>
+      </c>
+      <c r="H51" s="12">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="I51" s="22" t="s">
+        <v>183</v>
+      </c>
+      <c r="J51" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="K51" s="14"/>
+      <c r="L51" s="14"/>
+      <c r="M51" s="14"/>
+      <c r="N51" s="14"/>
+      <c r="O51" s="14"/>
+      <c r="P51" s="14"/>
+      <c r="Q51" s="14"/>
+      <c r="R51" s="26"/>
+    </row>
+    <row r="52" spans="1:18" ht="15">
+      <c r="A52" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="B52" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="C52" s="24" t="s">
+        <v>190</v>
+      </c>
+      <c r="D52" s="24" t="s">
+        <v>191</v>
+      </c>
+      <c r="E52" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="F52" s="25">
+        <v>46296</v>
+      </c>
+      <c r="G52" s="25">
+        <v>46310</v>
+      </c>
+      <c r="H52" s="12">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="I52" s="22" t="s">
+        <v>183</v>
+      </c>
+      <c r="J52" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="K52" s="14"/>
+      <c r="L52" s="14"/>
+      <c r="M52" s="14"/>
+      <c r="N52" s="14"/>
+      <c r="O52" s="14"/>
+      <c r="P52" s="14"/>
+      <c r="Q52" s="14"/>
+      <c r="R52" s="26"/>
+    </row>
+    <row r="54" spans="1:18" ht="18">
+      <c r="B54" s="27" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="55" spans="1:18" ht="15.5">
       <c r="B55" s="28" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="C55" s="29">
-        <f>COUNTIF(J6:J50,"進行中")</f>
-        <v>0</v>
+        <f>COUNTA(A6:A52)</f>
+        <v>47</v>
       </c>
     </row>
     <row r="56" spans="1:18" ht="15.5">
       <c r="B56" s="28" t="s">
-        <v>183</v>
+        <v>30</v>
       </c>
       <c r="C56" s="29">
-        <f>COUNTIF(J6:J50,"完了")</f>
-        <v>0</v>
+        <f>COUNTIF(J6:J52,"未着手")</f>
+        <v>47</v>
       </c>
     </row>
     <row r="57" spans="1:18" ht="15.5">
       <c r="B57" s="28" t="s">
-        <v>184</v>
-      </c>
-      <c r="C57" s="30">
-        <f>IFERROR(C56/C53,0)</f>
+        <v>194</v>
+      </c>
+      <c r="C57" s="29">
+        <f>COUNTIF(J6:J52,"進行中")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18" ht="15.5">
+      <c r="B58" s="28" t="s">
+        <v>195</v>
+      </c>
+      <c r="C58" s="29">
+        <f>COUNTIF(J6:J52,"完了")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18" ht="15.5">
+      <c r="B59" s="28" t="s">
+        <v>196</v>
+      </c>
+      <c r="C59" s="30">
+        <f>IFERROR(C58/C55,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3361,7 +3488,7 @@
   </mergeCells>
   <phoneticPr fontId="13"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="J6:J50" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="J6:J52" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"未着手,進行中,完了,保留"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3385,84 +3512,84 @@
   <sheetData>
     <row r="1" spans="1:3" ht="22.5">
       <c r="A1" s="31" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.5">
       <c r="A3" s="32" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="B3" s="32" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15">
       <c r="A4" s="8" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C4" s="34" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="15">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="30">
       <c r="A5" s="8" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="C5" s="34" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15">
       <c r="A6" s="8" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="C6" s="34" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15">
       <c r="A7" s="8" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="C7" s="34" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15">
       <c r="A8" s="8" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="C8" s="34" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15">
       <c r="A9" s="8" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="C9" s="34" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -3477,7 +3604,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -3487,138 +3614,152 @@
   <sheetData>
     <row r="1" spans="1:4" ht="22.5">
       <c r="A1" s="31" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16.5">
       <c r="A3" s="32" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="B3" s="32" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="D3" s="32" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="30">
       <c r="A4" s="33" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="B4" s="35" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="C4" s="34" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="D4" s="34" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="30">
       <c r="A5" s="33" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="C5" s="34" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="D5" s="34" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30">
       <c r="A6" s="33" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="C6" s="34" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="D6" s="34" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="30">
       <c r="A7" s="33" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="C7" s="34" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="D7" s="34" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30">
       <c r="A8" s="33" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="C8" s="34" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="D8" s="34" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30">
       <c r="A9" s="33" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="C9" s="34" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="D9" s="34" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="30">
       <c r="A10" s="33" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="D10" s="34" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="30">
       <c r="A11" s="33" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="C11" s="34" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="D11" s="34" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.5">
-      <c r="A14" s="36" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="45">
+      <c r="A12" s="33" t="s">
+        <v>249</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>237</v>
+      </c>
+      <c r="C12" s="34" t="s">
+        <v>250</v>
+      </c>
+      <c r="D12" s="34" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.5">
+      <c r="A15" s="36" t="s">
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>